<commit_message>
Update output Excel files with latest scraped data (2026-06-04)
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/featured.xlsx
+++ b/output/featured.xlsx
@@ -421,12 +421,12 @@
   <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="31" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
     <col width="8" customWidth="1" min="4" max="4"/>
-    <col width="45" customWidth="1" min="5" max="5"/>
-    <col width="47" customWidth="1" min="6" max="6"/>
+    <col width="55" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -470,7 +470,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Momacu</t>
+          <t>KD: The Devil</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -480,7 +480,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>All</t>
+          <t>Telugu</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -488,14 +488,10 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>featured/1/Momacu.jpg</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=ebWqjLUBgqE</t>
-        </is>
-      </c>
+          <t>featured/06-04-2026/KD The Devil.jpg</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
           <t>2026-06-04</t>
@@ -505,7 +501,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Maa Behen</t>
+          <t>29</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -515,7 +511,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>All</t>
+          <t>Telugu</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -523,14 +519,10 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>featured/1/Maa Behen.jpg</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=xYbLpsEhcfA</t>
-        </is>
-      </c>
+          <t>featured/06-04-2026/29.jpg</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
           <t>2026-06-04</t>
@@ -540,17 +532,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Premam Madhuram</t>
+          <t>Peddi</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Kannada</t>
+          <t>Telugu</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -558,14 +550,10 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>featured/1/Premam Madhuram.jpg</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=RkMt3-2m2mw</t>
-        </is>
-      </c>
+          <t>featured/06-04-2026/Peddi.jpg</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
           <t>2026-06-04</t>
@@ -575,7 +563,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Carmeni Selvam</t>
+          <t>Patriot</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -585,7 +573,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Tamil</t>
+          <t>Telugu</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -593,14 +581,10 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>featured/1/Carmeni Selvam.jpg</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=W4BLjlRo4Bs</t>
-        </is>
-      </c>
+          <t>featured/06-04-2026/Patriot.jpg</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
           <t>2026-06-04</t>
@@ -610,17 +594,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Beast of War</t>
+          <t>Sattendru Maarudhu Vaanilai</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>All</t>
+          <t>Tamil</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -628,14 +612,10 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>featured/1/Beast of War.jpg</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=x4Dk6joTDRg</t>
-        </is>
-      </c>
+          <t>featured/06-04-2026/Sattendru Maarudhu Vaanilai.jpg</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
           <t>2026-06-04</t>
@@ -645,7 +625,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Carmeni Selvam</t>
+          <t>Patriot</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -655,7 +635,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Telugu</t>
+          <t>Malayalam</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -663,14 +643,10 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>featured/1/Carmeni Selvam.jpg</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=ZmPVwT_R_eI</t>
-        </is>
-      </c>
+          <t>featured/06-04-2026/Patriot.jpg</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr">
         <is>
           <t>2026-06-04</t>
@@ -680,12 +656,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Rescue Dawn</t>
+          <t>Momacu</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2006</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -698,14 +674,10 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>featured/1/Rescue Dawn.jpg</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=UNm9Tzo5rvI</t>
-        </is>
-      </c>
+          <t>featured/06-04-2026/Momacu.jpg</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr">
         <is>
           <t>2026-06-04</t>
@@ -715,17 +687,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Aaahladam</t>
+          <t>Maa Behen</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Malayalam</t>
+          <t>All</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -733,14 +705,10 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>featured/1/Aaahladam.jpg</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=ciF1rVqYX9E</t>
-        </is>
-      </c>
+          <t>featured/06-04-2026/Maa Behen.jpg</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr">
         <is>
           <t>2026-06-04</t>
@@ -750,17 +718,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Trikala: Script of God</t>
+          <t>Premam Madhuram</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Telugu</t>
+          <t>Kannada</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -768,14 +736,10 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>featured/1/Trikala Script of God.jpg</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=U098Oyg8nYo</t>
-        </is>
-      </c>
+          <t>featured/06-04-2026/Premam Madhuram.jpg</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr">
         <is>
           <t>2026-06-04</t>
@@ -785,7 +749,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Blast Zone</t>
+          <t>Carmeni Selvam</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -795,7 +759,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Telugu</t>
+          <t>Tamil</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -803,14 +767,10 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>featured/1/Blast Zone.jpg</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=_vbRwxitX2o</t>
-        </is>
-      </c>
+          <t>featured/06-04-2026/Carmeni Selvam.jpg</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
           <t>2026-06-04</t>
@@ -820,17 +780,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Kattalan</t>
+          <t>Beast of War</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Telugu</t>
+          <t>All</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -838,14 +798,10 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>featured/1/Kattalan.jpg</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=iQMvxXmCk9I</t>
-        </is>
-      </c>
+          <t>featured/06-04-2026/Beast of War.jpg</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr">
         <is>
           <t>2026-06-04</t>
@@ -855,7 +811,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Sandigdham</t>
+          <t>Carmeni Selvam</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -873,14 +829,10 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>featured/1/Sandigdham.jpg</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=wTYXAINrYkw</t>
-        </is>
-      </c>
+          <t>featured/06-04-2026/Carmeni Selvam.jpg</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
           <t>2026-06-04</t>
@@ -890,12 +842,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>The Exorcism Of Emily Rose</t>
+          <t>Rescue Dawn</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2005</t>
+          <t>2006</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -908,14 +860,10 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>featured/1/The Exorcism Of Emily Rose.jpg</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=Bi-PLwxwvy8</t>
-        </is>
-      </c>
+          <t>featured/06-04-2026/Rescue Dawn.jpg</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
           <t>2026-06-04</t>
@@ -925,17 +873,17 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Kattalan</t>
+          <t>Aaahladam</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2026</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Hindi</t>
+          <t>Malayalam</t>
         </is>
       </c>
       <c r="D15" t="n">
@@ -943,14 +891,10 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>featured/1/Kattalan.jpg</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=iQMvxXmCk9I</t>
-        </is>
-      </c>
+          <t>featured/06-04-2026/Aaahladam.jpg</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
           <t>2026-06-04</t>
@@ -960,7 +904,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Purushaha</t>
+          <t>Trikala: Script of God</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -978,14 +922,10 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>featured/1/Purushaha.jpg</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=xs_NcJrsVy8</t>
-        </is>
-      </c>
+          <t>featured/06-04-2026/Trikala Script of God.jpg</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
           <t>2026-06-04</t>
@@ -995,7 +935,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Faces</t>
+          <t>Blast Zone</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -1005,7 +945,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>All</t>
+          <t>Telugu</t>
         </is>
       </c>
       <c r="D17" t="n">
@@ -1013,14 +953,10 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>featured/1/Faces.jpg</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>https://www.youtube.com/watch?v=6IxPD-jNdwM</t>
-        </is>
-      </c>
+          <t>featured/06-04-2026/Blast Zone.jpg</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr">
         <is>
           <t>2026-06-04</t>

</xml_diff>

<commit_message>
Add malayalam module, fix browser JS challenge, update docs
- New malayalam command scrapes https://www.5movierulz.discount/category/malayalam-featured
- Date-wise image folders (downloads/malayalam/MM-DD-YYYY/) same as home/featured
- Custom _page_url in malayalam.py handles no-trailing-slash requirement of .discount domain
- browser.py waits for #main selector to resolve JS challenge pages on paginated URLs
- Daily Summary tab now sorted newest date first across all modules
- DEFAULT_MALAYALAM_BASE_URL added to modules/config.py
- README and RUN.md updated with malayalam usage, updated default URLs section

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/output/featured.xlsx
+++ b/output/featured.xlsx
@@ -418,7 +418,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:G27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="31" customWidth="1" min="1" max="1"/>
@@ -426,7 +426,7 @@
     <col width="13" customWidth="1" min="3" max="3"/>
     <col width="8" customWidth="1" min="4" max="4"/>
     <col width="55" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="47" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -470,7 +470,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>KD: The Devil</t>
+          <t>Peter</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -480,7 +480,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Telugu</t>
+          <t>Kannada</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -488,20 +488,24 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>featured/06-04-2026/KD The Devil.jpg</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr"/>
+          <t>featured/06-05-2026/Peter.jpg</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=647TsP9EP-0</t>
+        </is>
+      </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>The Rise of Ashoka</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -511,7 +515,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Telugu</t>
+          <t>Tamil</t>
         </is>
       </c>
       <c r="D3" t="n">
@@ -519,20 +523,24 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>featured/06-04-2026/29.jpg</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr"/>
+          <t>featured/06-05-2026/The Rise of Ashoka.jpg</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=k4X8z0hWQ4I</t>
+        </is>
+      </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Peddi</t>
+          <t>Ugly Story</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -542,7 +550,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Telugu</t>
+          <t>Hindi</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -550,20 +558,24 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>featured/06-04-2026/Peddi.jpg</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr"/>
+          <t>featured/06-05-2026/Ugly Story.jpg</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=7hLQtxlhmeM</t>
+        </is>
+      </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Patriot</t>
+          <t>The Rise of Ashoka</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -573,7 +585,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Telugu</t>
+          <t>Kannada</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -581,20 +593,24 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>featured/06-04-2026/Patriot.jpg</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr"/>
+          <t>featured/06-05-2026/The Rise of Ashoka.jpg</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=k4X8z0hWQ4I</t>
+        </is>
+      </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Sattendru Maarudhu Vaanilai</t>
+          <t>Office Romance</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -604,7 +620,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Tamil</t>
+          <t>All</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -612,20 +628,24 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>featured/06-04-2026/Sattendru Maarudhu Vaanilai.jpg</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr"/>
+          <t>featured/06-05-2026/Office Romance.jpg</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=M7KrcId8LQg</t>
+        </is>
+      </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Patriot</t>
+          <t>The Marked Woman</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -635,7 +655,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Malayalam</t>
+          <t>All</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -643,20 +663,24 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>featured/06-04-2026/Patriot.jpg</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr"/>
+          <t>featured/06-05-2026/The Marked Woman.jpg</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=161b4xLkokE</t>
+        </is>
+      </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Momacu</t>
+          <t>Ugly Story</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -666,7 +690,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>All</t>
+          <t>Tamil</t>
         </is>
       </c>
       <c r="D8" t="n">
@@ -674,20 +698,24 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>featured/06-04-2026/Momacu.jpg</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr"/>
+          <t>featured/06-05-2026/Ugly Story.jpg</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=7hLQtxlhmeM</t>
+        </is>
+      </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Maa Behen</t>
+          <t>Sukhamano Sukhamann</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -697,7 +725,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>All</t>
+          <t>Malayalam</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -705,30 +733,34 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>featured/06-04-2026/Maa Behen.jpg</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr"/>
+          <t>featured/06-05-2026/Sukhamano Sukhamann.jpg</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=YiYDvpWNK3o</t>
+        </is>
+      </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Premam Madhuram</t>
+          <t>The Rise of Ashoka</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Kannada</t>
+          <t>Telugu</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -736,20 +768,24 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>featured/06-04-2026/Premam Madhuram.jpg</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr"/>
+          <t>featured/06-05-2026/The Rise of Ashoka.jpg</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=k4X8z0hWQ4I</t>
+        </is>
+      </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Carmeni Selvam</t>
+          <t>Ugly Story</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -759,7 +795,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Tamil</t>
+          <t>Telugu</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -767,30 +803,34 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>featured/06-04-2026/Carmeni Selvam.jpg</t>
-        </is>
-      </c>
-      <c r="F11" t="inlineStr"/>
+          <t>featured/06-05-2026/Ugly Story.jpg</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=7hLQtxlhmeM</t>
+        </is>
+      </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Beast of War</t>
+          <t>KD: The Devil</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>All</t>
+          <t>Telugu</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -798,10 +838,9 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>featured/06-04-2026/Beast of War.jpg</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr"/>
+          <t>featured/06-04-2026/KD The Devil.jpg</t>
+        </is>
+      </c>
       <c r="G12" t="inlineStr">
         <is>
           <t>2026-06-04</t>
@@ -811,7 +850,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Carmeni Selvam</t>
+          <t>29</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -829,10 +868,9 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>featured/06-04-2026/Carmeni Selvam.jpg</t>
-        </is>
-      </c>
-      <c r="F13" t="inlineStr"/>
+          <t>featured/06-04-2026/29.jpg</t>
+        </is>
+      </c>
       <c r="G13" t="inlineStr">
         <is>
           <t>2026-06-04</t>
@@ -842,17 +880,17 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Rescue Dawn</t>
+          <t>Peddi</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2006</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>All</t>
+          <t>Telugu</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -860,10 +898,9 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>featured/06-04-2026/Rescue Dawn.jpg</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr"/>
+          <t>featured/06-04-2026/Peddi.jpg</t>
+        </is>
+      </c>
       <c r="G14" t="inlineStr">
         <is>
           <t>2026-06-04</t>
@@ -873,17 +910,17 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Aaahladam</t>
+          <t>Patriot</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>2026</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Malayalam</t>
+          <t>Telugu</t>
         </is>
       </c>
       <c r="D15" t="n">
@@ -891,10 +928,9 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>featured/06-04-2026/Aaahladam.jpg</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr"/>
+          <t>featured/06-04-2026/Patriot.jpg</t>
+        </is>
+      </c>
       <c r="G15" t="inlineStr">
         <is>
           <t>2026-06-04</t>
@@ -904,7 +940,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Trikala: Script of God</t>
+          <t>Sattendru Maarudhu Vaanilai</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -914,7 +950,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Telugu</t>
+          <t>Tamil</t>
         </is>
       </c>
       <c r="D16" t="n">
@@ -922,10 +958,9 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>featured/06-04-2026/Trikala Script of God.jpg</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr"/>
+          <t>featured/06-04-2026/Sattendru Maarudhu Vaanilai.jpg</t>
+        </is>
+      </c>
       <c r="G16" t="inlineStr">
         <is>
           <t>2026-06-04</t>
@@ -935,29 +970,328 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
+          <t>Patriot</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Malayalam</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>1</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>featured/06-04-2026/Patriot.jpg</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Momacu</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>1</v>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>featured/06-04-2026/Momacu.jpg</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Maa Behen</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>1</v>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>featured/06-04-2026/Maa Behen.jpg</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Premam Madhuram</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Kannada</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>1</v>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>featured/06-04-2026/Premam Madhuram.jpg</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Carmeni Selvam</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Tamil</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>1</v>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>featured/06-04-2026/Carmeni Selvam.jpg</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Beast of War</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>1</v>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>featured/06-04-2026/Beast of War.jpg</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Carmeni Selvam</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Telugu</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>1</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>featured/06-04-2026/Carmeni Selvam.jpg</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Rescue Dawn</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>2006</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>1</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>featured/06-04-2026/Rescue Dawn.jpg</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Aaahladam</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Malayalam</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>1</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>featured/06-04-2026/Aaahladam.jpg</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Trikala: Script of God</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Telugu</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>1</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>featured/06-04-2026/Trikala Script of God.jpg</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
           <t>Blast Zone</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>2026</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
         <is>
           <t>Telugu</t>
         </is>
       </c>
-      <c r="D17" t="n">
-        <v>1</v>
-      </c>
-      <c r="E17" t="inlineStr">
+      <c r="D27" t="n">
+        <v>1</v>
+      </c>
+      <c r="E27" t="inlineStr">
         <is>
           <t>featured/06-04-2026/Blast Zone.jpg</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr">
+      <c r="G27" t="inlineStr">
         <is>
           <t>2026-06-04</t>
         </is>
@@ -974,7 +1308,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -996,10 +1330,20 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B2" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
         <v>16</v>
       </c>
     </row>

</xml_diff>